<commit_message>
Daily scrape output - 2026-06-24
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_current.xlsx
+++ b/outputs/pinnacle_corners_current.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,80 +454,626 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46196</v>
+        <v>46201</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10.69</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10.35</v>
+        <v>9.57</v>
       </c>
       <c r="F3" t="n">
-        <v>1.96</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46196</v>
+        <v>46200</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>Cape Verde</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.859999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="F4" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Curacao</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-4.48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.53</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.58</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-3.02</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-3.61</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-1.53</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-4.21</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-2.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-1.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-3.73</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Turkiye</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-2.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-06-25
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_current.xlsx
+++ b/outputs/pinnacle_corners_current.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,33 +454,33 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46201</v>
+        <v>46198</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8.300000000000001</v>
+        <v>10.24</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.03</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46197</v>
+        <v>46201</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -489,19 +489,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>9.57</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>2.92</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="4">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>8.69</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F4" t="n">
         <v>0.14</v>
@@ -550,10 +550,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9.210000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="F5" t="n">
-        <v>-1.04</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="6">
@@ -602,15 +602,15 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>9.390000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="F7" t="n">
-        <v>-4.48</v>
+        <v>-4.47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -619,24 +619,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>DR Congo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Uzbekistan</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>8.83</v>
+        <v>8.82</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.53</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46200</v>
+        <v>46198</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -645,24 +645,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DR Congo</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>8.81</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>1.15</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -671,24 +671,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>9.539999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.58</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46200</v>
+        <v>46198</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -697,24 +697,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>8.1</v>
+        <v>9.31</v>
       </c>
       <c r="F11" t="n">
-        <v>0.41</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -723,24 +723,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>9.369999999999999</v>
+        <v>8.74</v>
       </c>
       <c r="F12" t="n">
-        <v>0.93</v>
+        <v>-3.02</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -749,24 +749,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8.74</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.02</v>
+        <v>-3.61</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -775,19 +775,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8.92</v>
+        <v>9.65</v>
       </c>
       <c r="F14" t="n">
-        <v>2.95</v>
+        <v>-1.51</v>
       </c>
     </row>
     <row r="15">
@@ -801,19 +801,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>England</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>10.09</v>
       </c>
       <c r="F15" t="n">
-        <v>-3.61</v>
+        <v>-4.19</v>
       </c>
     </row>
     <row r="16">
@@ -827,24 +827,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>9.67</v>
+        <v>7.82</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.53</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -853,24 +853,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>10.09</v>
+        <v>9.18</v>
       </c>
       <c r="F17" t="n">
-        <v>-4.21</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -879,24 +879,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>7.8</v>
+        <v>9.25</v>
       </c>
       <c r="F18" t="n">
-        <v>0.36</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -905,24 +905,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Turkiye</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>8.720000000000001</v>
+        <v>9.58</v>
       </c>
       <c r="F19" t="n">
-        <v>-2.9</v>
+        <v>-0.89</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -931,148 +931,18 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>9.16</v>
+        <v>9.51</v>
       </c>
       <c r="F20" t="n">
-        <v>2.66</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>8.15</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-1.2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>9.02</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-0.19</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>9.609999999999999</v>
-      </c>
-      <c r="F23" t="n">
-        <v>-3.73</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Turkiye</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>9.52</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.65</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>9.51</v>
-      </c>
-      <c r="F25" t="n">
         <v>-2.23</v>
       </c>
     </row>

</xml_diff>